<commit_message>
chore: update ticket prices
</commit_message>
<xml_diff>
--- a/ticket_prices.xlsx
+++ b/ticket_prices.xlsx
@@ -7,10 +7,16 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="横浜FM-鹿島_807" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="川崎-京都サンガＦ．Ｃ．_815" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="名古屋-清水_808" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="東京V-柏_814" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="横浜FM_808" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="FC東京_823" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="水戸_807" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="浦和_815" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="千葉_808" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="川崎F_815" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="柏_808" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="町田_829" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="鹿島_814" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="東京V_821" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,199 +433,417 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>バックアッパー(ホーム)３層</t>
+          <t>アウェイゴール裏自由</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>バックＳＢ １層(ホーム)</t>
+          <t>アビスパシート指定</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>バックＳＢ ２層(ホーム)</t>
+          <t>ウェルカムシート自由</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>バックＳＣ １層(ホーム)</t>
+          <t>エキサイティングシート指定</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>バックＳＣ １層(ミックス)</t>
+          <t>バックスタンド自由（Ｂ１）</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>バックＳＣ ２層(ホーム)</t>
+          <t>バックスタンド自由（Ｂ７）</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>バックＳＣ ２層(ミックス)</t>
+          <t>ピッチサイドシート指定（Ｂ２）</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>ビジターサポーターズシート１層</t>
+          <t>ピッチサイドシート指定（Ｂ６）</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>ビジターサポーターズシート２層</t>
+          <t>プレミアムシート指定</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>ホームサポーターズシート１層</t>
+          <t>ホームゴール裏自由</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>ホームサポーターズシート２層</t>
+          <t>メインスタンド指定（Ｍ１）</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>ホームパノラマシート３層</t>
+          <t>メインスタンド指定（Ｍ２）</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>ミックスパノラマシート３層</t>
+          <t>メインスタンド指定（Ｍ５）</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>メインＳＡ ３層(ホーム)</t>
+          <t>メインスタンド指定（Ｍ６）</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>メインＳＡ ３層(ミックス)</t>
+          <t>メインスタンド自由（Ｍ１）</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>メインＳＳ １層(ホーム)</t>
+          <t>メインスタンド自由（Ｍ６）</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>メインＳＳ １層(ミックス)</t>
+          <t>柴田産業Axion指定</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>メインＳＳ ２層(ホーム)</t>
+          <t>車いす席　平面駐車場付</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>メインＳＳ ２層(ミックス)</t>
+          <t>車いす席　立体駐車場付</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-26 10:09</t>
+          <t>2026-07-26 10:18</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>4,600</t>
+          <t>4,000</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>13,400</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2,000</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>7,800</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>4,000</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>4,000</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>5,800</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>5,800</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>15,800</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>3,300</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>7,300</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>8,300</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>9,100</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>6,900</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>4,500</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>4,000</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>4,700</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>4,000 完売</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>4,000 完売</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>checked_at</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>クッション付きシート　北側</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>クッション付きシート　南側</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>セブン-イレブンシート</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>バック</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>バックセンター</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>バックセンターＵＦ</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>バックＵＦ</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>ビジター</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>ホーム</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>ホームＵＦ</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>メイン上層</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>メインＳ　北側</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>メインＳ　南側</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>メインＳＳ　北側</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>メインＳＳ　南側</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>メインＳＳＳ</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>ユニバーサル席　代表者</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>ユニバーサル席　同伴者</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>南サイド</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-26 10:18</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>11,500</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>11,500</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>5,400</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>6,000</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>6,000</t>
+          <t>4,000</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>6,200 完売</t>
+          <t>5,400</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>6,200</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>5,400</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>6,000 完売</t>
-        </is>
-      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>4,800</t>
+          <t>4,100</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>4,800 完売</t>
+          <t>3,900</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>4,600 完売</t>
+          <t>4,700</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4,200</t>
+          <t>5,000</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>3,800</t>
+          <t>6,300</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>4,400</t>
+          <t>6,300</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>5,000</t>
+          <t>8,700</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>5,800</t>
+          <t>8,700</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>7,400</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>8,200 完売</t>
+          <t>4,000</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>7,000</t>
+          <t>4,000</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>8,200 完売</t>
+          <t>3,900</t>
         </is>
       </c>
     </row>
@@ -634,7 +858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD2"/>
+  <dimension ref="A1:U2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -645,299 +869,209 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>ごちクルグループシート６</t>
+          <t>カテゴリー１北（１層）</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>グループシート４</t>
+          <t>カテゴリー１南（１層）</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>セブンイレブンピッチサイド席</t>
+          <t>カテゴリー２北（１層）</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>テーブル付ペアシート</t>
+          <t>カテゴリー２南（１層）</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>バック車椅子席</t>
+          <t>カテゴリー３（１層）</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>バックＳ指定北側</t>
+          <t>カテゴリー３（２層）</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>バックＳ指定南側</t>
+          <t>カテゴリー４北（１層）</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>バックＳＳ指定</t>
+          <t>カテゴリー４北（２層）</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>ビジターＡ自由</t>
+          <t>カテゴリー４南（１層）</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>ビジターＳ指定</t>
+          <t>カテゴリー４南（２層）</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>ビジターＳＡ指定</t>
+          <t>カテゴリー５</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>ファミリーシート３</t>
+          <t>ゼルビアサポーターズシート立見席</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>ファミリーシート４</t>
+          <t>バック上層（３層）自由席</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>ファミリーシート６</t>
+          <t>ビジターサポーターズシート指定席</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>ペアシート北側</t>
+          <t>プレミアムシート(ラウンジ付)</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>ペアシート南側</t>
+          <t>プレミアムシート（２層）</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>ホームＡ指定</t>
+          <t>メイン上層（２層）</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>ホームＡ自由</t>
+          <t>メイン上層（３層）</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>メイン車椅子席</t>
+          <t>南サイド（２・３層）</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>メインＳ指定北側</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>メインＳ指定南側</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>メインＳＳ指定上層中央</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>メインＳＳ指定下層北側</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>メインＳＳ指定下層南側</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>ＳＡ指定北側</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>ＳＡ指定南側</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>ＳＧ指定</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>ＳＳＳ指定</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>ＴＨＥＲＭＯＳ パーティーシート</t>
+          <t>車椅子同行者席</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-26 10:09</t>
+          <t>2026-07-26 10:18</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>7,200 完売</t>
+          <t>8,400</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6,000 完売</t>
+          <t>8,400</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>6,000 完売</t>
+          <t>7,800</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>7,000</t>
+          <t>7,800</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>3,500</t>
+          <t>7,400</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>6,400 完売</t>
+          <t>8,400</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>5,800</t>
+          <t>6,600</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>7,000 完売</t>
+          <t>6,600</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>3,700 完売</t>
+          <t>6,600</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>6,400 完売</t>
+          <t>6,600</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>4,700 完売</t>
+          <t>3,300</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>6,000 完売</t>
+          <t>4,000</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>6,000 完売</t>
+          <t>3,600</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>6,000 完売</t>
+          <t>4,100</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>7,100 完売</t>
+          <t>23,500</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>6,700 完売</t>
+          <t>12,100</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
+          <t>6,900</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
           <t>4,200</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>3,600</t>
-        </is>
-      </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>4,400</t>
+          <t>3,400</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>6,600 完売</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>6,100</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>7,400 完売</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>7,800 完売</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>7,400 完売</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>4,600 完売</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>4,200</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>5,300 完売</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>8,700 完売</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>7,700 完売</t>
+          <t>7,700</t>
         </is>
       </c>
     </row>
@@ -952,7 +1086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:T3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -963,77 +1097,97 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>アウェイ指定席</t>
+          <t>バックアッパー(ホーム)３層</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>ゴール裏指定席１階北側</t>
+          <t>バックＳＢ １層(ホーム)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>ゴール裏指定席１階南側</t>
+          <t>バックＳＢ ２層(ホーム)</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>ゴール裏指定席２階北側</t>
+          <t>バックＳＣ １層(ホーム)</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>セブン-イレブン最前列シート</t>
+          <t>バックＳＣ １層(ミックス)</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>バック３階指定席</t>
+          <t>バックＳＣ ２層(ホーム)</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>バック４階指定席</t>
+          <t>バックＳＣ ２層(ミックス)</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>メイン３階指定席</t>
+          <t>ビジターサポーターズシート１層</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>メイン４階指定席</t>
+          <t>ビジターサポーターズシート２層</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>ロイヤルシート</t>
+          <t>ホームサポーターズシート１層</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>Ａ指定席</t>
+          <t>ホームサポーターズシート２層</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>Ｂ指定席</t>
+          <t>ホームパノラマシート３層</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>Ｃ指定席</t>
+          <t>ミックスパノラマシート３層</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>Ｓ指定席</t>
+          <t>メインＳＡ ３層(ホーム)</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>ＳＳ指定席</t>
+          <t>メインＳＡ ３層(ミックス)</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>メインＳＳ １層(ホーム)</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>メインＳＳ １層(ミックス)</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>メインＳＳ ２層(ホーム)</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>メインＳＳ ２層(ミックス)</t>
         </is>
       </c>
     </row>
@@ -1045,77 +1199,199 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>4,600</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>5,400</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>6,000</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>6,000</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>6,200 完売</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>5,400</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>6,000 完売</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>4,800</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>4,800 完売</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>4,600 完売</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>4,200</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>3,800</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>4,400</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
           <t>5,000</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>5,000 完売</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>5,800</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>7,400</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>8,200 完売</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>7,000</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>8,200 完売</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-26 10:18</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>4,600</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>5,400</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>6,000</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>6,000</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>6,200 完売</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>5,400</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>6,000 完売</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>4,800</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>4,800 完売</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>4,600 完売</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
         <is>
           <t>4,200</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>4,600</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>9,200</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>4,800</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>3,000</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>5,200</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>3,200</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>12,000 完売</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>7,200</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>7,200</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>3,800</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>8,200</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>9,600</t>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>4,400</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>5,000</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>5,800</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>7,400</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>8,200 完売</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>7,000</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>8,200 完売</t>
         </is>
       </c>
     </row>
@@ -1130,7 +1406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:AD3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1141,87 +1417,147 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>ゴール裏ビジター指定</t>
+          <t>ごちクルグループシート６</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>ゴール裏ホーム自由</t>
+          <t>グループシート４</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>ゴール裏ホーム自由3層</t>
+          <t>セブンイレブンピッチサイド席</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>サイドミックス指定3層</t>
+          <t>テーブル付ペアシート</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>バックホーム指定</t>
+          <t>バック車椅子席</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>バックホーム指定3層</t>
+          <t>バックＳ指定北側</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>バックホーム指定センター</t>
+          <t>バックＳ指定南側</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>バックミックス指定</t>
+          <t>バックＳＳ指定</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>バックミックス指定3層</t>
+          <t>ビジターＡ自由</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>プレミアムシートホームラウンジ付</t>
+          <t>ビジターＳ指定</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>プレミアムシートミックスラウンジ付</t>
+          <t>ビジターＳＡ指定</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>メインSS指定ホーム</t>
+          <t>ファミリーシート３</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>メインSS指定ミックス</t>
+          <t>ファミリーシート４</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>メインS指定ホーム</t>
+          <t>ファミリーシート６</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>メインS指定ミックス</t>
+          <t>ペアシート北側</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>メイン指定ホーム3層</t>
+          <t>ペアシート南側</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>メイン指定ミックス3層</t>
+          <t>ホームＡ指定</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>ホームＡ自由</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>メイン車椅子席</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>メインＳ指定北側</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>メインＳ指定南側</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>メインＳＳ指定上層中央</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>メインＳＳ指定下層北側</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>メインＳＳ指定下層南側</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>ＳＡ指定北側</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>ＳＡ指定南側</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>ＳＧ指定</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>ＳＳＳ指定</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>ＴＨＥＲＭＯＳ パーティーシート</t>
         </is>
       </c>
     </row>
@@ -1233,6 +1569,1260 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>7,200 完売</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>6,000 完売</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>6,000 完売</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>7,000</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>3,500</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>6,400 完売</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>5,800</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>7,000 完売</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>3,700 完売</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>6,400 完売</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>4,700 完売</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>6,000 完売</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>6,000 完売</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>6,000 完売</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>7,100 完売</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>6,700 完売</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>4,200</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>3,600</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>4,400</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>6,600 完売</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>6,100</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>7,400 完売</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>7,800 完売</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>7,400 完売</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>4,600 完売</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>4,200</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>5,300 完売</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>8,700 完売</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>7,700 完売</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-26 10:18</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>7,200 完売</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>6,000 完売</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>6,000 完売</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>7,000</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>3,500</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>6,400 完売</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>5,800</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>7,000 完売</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>3,700 完売</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>6,400 完売</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>4,700 完売</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>6,000 完売</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>6,000 完売</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>6,000 完売</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>7,100 完売</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>6,700 完売</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>4,200</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>3,600</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>4,400</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>6,600 完売</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>6,100</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>7,400 完売</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>7,800 完売</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>7,400 完売</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>4,600 完売</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>4,200</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>5,300 完売</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>8,700 完売</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>7,700 完売</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>checked_at</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>アウェイ指定席</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>ゴール裏指定席１階北側</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>ゴール裏指定席１階南側</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>ゴール裏指定席２階北側</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>セブン-イレブン最前列シート</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>バック３階指定席</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>バック４階指定席</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>メイン３階指定席</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>メイン４階指定席</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>ロイヤルシート</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Ａ指定席</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Ｂ指定席</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Ｃ指定席</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Ｓ指定席</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>ＳＳ指定席</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-26 10:09</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>5,000</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>5,000 完売</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>4,200</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>4,600</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>9,200</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>4,800</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>3,000</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>5,200</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>3,200</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>12,000 完売</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>7,200</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>7,200</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>3,800</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>8,200</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>9,600</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-26 10:18</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>5,000</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>5,000 完売</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>4,200</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>4,600</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>9,200</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>4,800</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>3,000</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>5,200</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>3,200</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>12,000 完売</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>7,200</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>7,200</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>3,800</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>8,200</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>9,600</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>checked_at</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>バック指定席（ホーム）</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>ビジター指定席</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>ホーム応援エリア席</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>メインミックス指定席</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Ｓ指定席　北</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Ｓ指定席　南</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>ＳＡ指定席</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>ＳＢ指定席</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>ＳＳ指定席</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-26 10:18</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>3,500</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>3,500</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>3,000</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>4,200</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>4,600</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>4,600</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>4,200</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>4,200</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>5,200</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AC2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>checked_at</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>エキサイティングシート(ホーム)前方</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>エキサイティングシート（ホーム）</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>バックセンターシート上段ホーム</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>バックセンターシート下段ホーム</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>バリュープライスシートAホーム</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>バリュープライスシートBホーム</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>ビジターサポーター指定席</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>ホームサポーター指定席</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>ホームサポーター自由席</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>ホームバック北A指定席上段</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ホームバック北A指定席下段</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>ホームバック北B指定席上段</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>ホームバック北B指定席下段</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>ホームバック南A指定席上段</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>ホームバック南A指定席下段</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>ホームバック南B指定席上段</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>ホームバック南B指定席下段</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>ホームメインセンターA指定席</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>ホームメイン北A指定席</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>ホームメイン北SS指定席</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>ホームメイン北SS指定席前方</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>ホームメイン北S指定席</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>ホームメイン北S指定席前方</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>ホームメイン南A指定席</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>ホームメイン南SS指定席</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>ホームメイン南SS指定席前方</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>ミックスメイン南S指定席</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>ミックスメイン南S指定席前方</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-26 10:18</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>13,800 完売</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>12,800 完売</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>5,000 完売</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>5,800 完売</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>3,500</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2,500 完売</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>3,800</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>3,500 完売</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>3,600</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>4,800</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>5,400 完売</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>4,200</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>5,000</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>4,200</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>5,000 完売</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>3,300</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>3,700</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>7,300 完売</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>5,700 完売</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>8,600 完売</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>9,600 完売</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>7,200</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>8,200 完売</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>6,000</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>8,900</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>9,900 完売</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>7,000 完売</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>8,000</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>checked_at</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>カテゴリー４</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>カテゴリー４ミックス</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>カテゴリー４ミックス視界制限席</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>カテゴリー４視界制限席</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>カテゴリー５</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>カテゴリー５視界制限席</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>カテゴリー６指定席</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>カテゴリー６自由席</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>ガンバサポーターシート</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>ビジター指定席</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>モリタにこにこ家族ラウンジ</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>車椅子ミックス席</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>車椅子席</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-26 10:18</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>4,000</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>4,000</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>3,500</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>3,500</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>3,400</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2,900</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2,900</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2,600</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>3,000</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>3,400</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>7,500</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>5,600</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>5,600</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>checked_at</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ゴール裏ビジター指定</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>ゴール裏ホーム自由</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>ゴール裏ホーム自由3層</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>サイドミックス指定3層</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>バックホーム指定</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>バックホーム指定3層</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>バックホーム指定センター</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>バックミックス指定</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>バックミックス指定3層</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>プレミアムシートホームラウンジ付</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>プレミアムシートミックスラウンジ付</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>メインSS指定ホーム</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>メインSS指定ミックス</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>メインS指定ホーム</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>メインS指定ミックス</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>メイン指定ホーム3層</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>メイン指定ミックス3層</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-26 10:09</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>4,500 [変動]</t>
         </is>
       </c>
@@ -1312,6 +2902,98 @@
         </is>
       </c>
       <c r="R2" t="inlineStr">
+        <is>
+          <t>5,600 [変動]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-26 10:18</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>4,500 [変動]</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>3,600</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>3,300</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>4,100 [変動]</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>4,400</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>3,900</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>4,900</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>6,100 [変動]</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>5,200 [変動]</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>13,500</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>14,600 [変動]</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>7,500</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>10,000 [変動]</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>6,500</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>8,800 [変動]</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>4,700</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
         <is>
           <t>5,600 [変動]</t>
         </is>

</xml_diff>